<commit_message>
Review workbook: the 138 installed SRVs still awaiting their Unit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVqNU2fQRYCLfmxh5xLgG1
</commit_message>
<xml_diff>
--- a/srv-unit-review.xlsx
+++ b/srv-unit-review.xlsx
@@ -11,7 +11,7 @@
     <sheet name="محتاجة Unit" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'محتاجة Unit'!$A$1:$K$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'محتاجة Unit'!$A$1:$K$139</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -451,7 +451,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>148</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3">
@@ -464,16 +464,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ريليفات محتاجة محطة</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    <row r="4"/>
     <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -489,257 +480,11 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>المحطة</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>عدد الريليفات</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>الدولفين</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>الشهداء</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>الخمايل</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>فويل اب الدائرى</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>المعصرة</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>عز الدين</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>العمرانية</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>مصدق</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>وادى حوف</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>شبين</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>الصحراوى</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>شبرا</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>بني سويف</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>دشلوط</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>حديقة بدر</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>بني سويف الجراج</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>قنا</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>الصفوة</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>المحور المركزى</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>الياسمين</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>حدائق اكتوبر</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>دائرى الهرم</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>زايد</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>سفنكس</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>3</v>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ريليفات Storage فويل اب الدائرى (3): قرار المالك تفضل على مستوى المحطة لأنها مشتركة بين الـ 2 Unit — سيبها فاضية.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -753,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K149"/>
+  <dimension ref="A1:K139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2845,33 +2590,38 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>الخمائل</t>
+          <t>الخمائل 2</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>264764</t>
+          <t>JTC-2102-1006</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>306 BAR</t>
+          <t>164.8 BAR</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
           <t>الخمايل 1 | الخمايل 2</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>الخمايل 2</t>
         </is>
       </c>
       <c r="I49" s="2" t="n"/>
       <c r="K49" t="inlineStr">
         <is>
-          <t>7bb3e8c7-aeeb-436b-b4af-102a85ae719b</t>
+          <t>5ac07e80-2474-440b-ac43-ddbabff56776</t>
         </is>
       </c>
     </row>
@@ -2888,33 +2638,38 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>الخمائل</t>
+          <t>الخمائل 1</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>264772</t>
+          <t>JTC-2102-1029</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>306 BAR</t>
+          <t>164.8 BAR</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
           <t>الخمايل 1 | الخمايل 2</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>الخمايل 1</t>
         </is>
       </c>
       <c r="I50" s="2" t="n"/>
       <c r="K50" t="inlineStr">
         <is>
-          <t>b091deaa-cf99-47e5-a006-b6da624d636e</t>
+          <t>2e6d60d4-4634-4ea8-8331-f49e8ac5452f</t>
         </is>
       </c>
     </row>
@@ -2931,33 +2686,38 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>الخمائل</t>
+          <t>الخمائل 1</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>264985</t>
+          <t>JTC-2102-1088</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>306 BAR</t>
+          <t>294.2 BAR</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
           <t>الخمايل 1 | الخمايل 2</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>الخمايل 1</t>
         </is>
       </c>
       <c r="I51" s="2" t="n"/>
       <c r="K51" t="inlineStr">
         <is>
-          <t>87a656f1-8fc2-462a-a53a-073c2b9daed5</t>
+          <t>b4f51e0d-9400-4a8c-86ca-bddcdf4ac5de</t>
         </is>
       </c>
     </row>
@@ -2974,7 +2734,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>الخمائل 1</t>
+          <t>الخمائل 2</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2984,12 +2744,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>JTC-2102-1029</t>
+          <t>JTC-2102-1118</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>164.8 BAR</t>
+          <t>32.4 BAR</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2999,13 +2759,13 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>الخمايل 1</t>
+          <t>الخمايل 2</t>
         </is>
       </c>
       <c r="I52" s="2" t="n"/>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2e6d60d4-4634-4ea8-8331-f49e8ac5452f</t>
+          <t>4012bcbc-f2c4-44c6-a885-92c25b9a823c</t>
         </is>
       </c>
     </row>
@@ -3032,12 +2792,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>JTC-2102-1088</t>
+          <t>JTC-2102-1148</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>294.2 BAR</t>
+          <t>32.4 BAR</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3053,7 +2813,7 @@
       <c r="I53" s="2" t="n"/>
       <c r="K53" t="inlineStr">
         <is>
-          <t>b4f51e0d-9400-4a8c-86ca-bddcdf4ac5de</t>
+          <t>652b3665-44eb-437e-a60d-63fe620f9b30</t>
         </is>
       </c>
     </row>
@@ -3070,7 +2830,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>الخمائل 1</t>
+          <t>الخمائل 2</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3080,12 +2840,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>JTC-2102-1148</t>
+          <t>JTC-2102-1179</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>32.4 BAR</t>
+          <t>65.7 BAR</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3095,13 +2855,13 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>الخمايل 1</t>
+          <t>الخمايل 2</t>
         </is>
       </c>
       <c r="I54" s="2" t="n"/>
       <c r="K54" t="inlineStr">
         <is>
-          <t>652b3665-44eb-437e-a60d-63fe620f9b30</t>
+          <t>7bd9f3f3-c17b-4cb2-83e9-6418269b38a6</t>
         </is>
       </c>
     </row>
@@ -3166,7 +2926,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>الخمائل 1</t>
+          <t>الخمائل 2</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3176,7 +2936,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>JTC-2102-1274</t>
+          <t>JTC-2102-1245</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3191,13 +2951,13 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>الخمايل 1</t>
+          <t>الخمايل 2</t>
         </is>
       </c>
       <c r="I56" s="2" t="n"/>
       <c r="K56" t="inlineStr">
         <is>
-          <t>cbabc3ca-6839-4557-a85f-b16dd1a5f252</t>
+          <t>533b33bc-6582-4346-ab7a-4c2391c3ab5c</t>
         </is>
       </c>
     </row>
@@ -3214,7 +2974,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>الخمائل 2</t>
+          <t>الخمائل 1</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3224,12 +2984,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>JTC-2102-1006</t>
+          <t>JTC-2102-1274</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>164.8 BAR</t>
+          <t>17.7 BAR</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3239,13 +2999,13 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>الخمايل 2</t>
+          <t>الخمايل 1</t>
         </is>
       </c>
       <c r="I57" s="2" t="n"/>
       <c r="K57" t="inlineStr">
         <is>
-          <t>5ac07e80-2474-440b-ac43-ddbabff56776</t>
+          <t>cbabc3ca-6839-4557-a85f-b16dd1a5f252</t>
         </is>
       </c>
     </row>
@@ -3272,12 +3032,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>JTC-2102-1118</t>
+          <t>JTC-2102-164</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>32.4 BAR</t>
+          <t>294.2 BAR</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3293,7 +3053,7 @@
       <c r="I58" s="2" t="n"/>
       <c r="K58" t="inlineStr">
         <is>
-          <t>4012bcbc-f2c4-44c6-a885-92c25b9a823c</t>
+          <t>e3aec884-a228-4b6d-a532-05fd65087a48</t>
         </is>
       </c>
     </row>
@@ -3310,38 +3070,33 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>الخمائل 2</t>
+          <t>الخمائل</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>JTC-2102-1179</t>
+          <t>264764</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>65.7 BAR</t>
+          <t>306 BAR</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
           <t>الخمايل 1 | الخمايل 2</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>الخمايل 2</t>
         </is>
       </c>
       <c r="I59" s="2" t="n"/>
       <c r="K59" t="inlineStr">
         <is>
-          <t>7bd9f3f3-c17b-4cb2-83e9-6418269b38a6</t>
+          <t>7bb3e8c7-aeeb-436b-b4af-102a85ae719b</t>
         </is>
       </c>
     </row>
@@ -3358,38 +3113,33 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>الخمائل 2</t>
+          <t>الخمائل</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>JTC-2102-1245</t>
+          <t>264772</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>17.7 BAR</t>
+          <t>306 BAR</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
           <t>الخمايل 1 | الخمايل 2</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>الخمايل 2</t>
         </is>
       </c>
       <c r="I60" s="2" t="n"/>
       <c r="K60" t="inlineStr">
         <is>
-          <t>533b33bc-6582-4346-ab7a-4c2391c3ab5c</t>
+          <t>b091deaa-cf99-47e5-a006-b6da624d636e</t>
         </is>
       </c>
     </row>
@@ -3406,38 +3156,33 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>الخمائل 2</t>
+          <t>الخمائل</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>JTC-2102-164</t>
+          <t>264985</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>294.2 BAR</t>
+          <t>306 BAR</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
           <t>الخمايل 1 | الخمايل 2</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>الخمايل 2</t>
         </is>
       </c>
       <c r="I61" s="2" t="n"/>
       <c r="K61" t="inlineStr">
         <is>
-          <t>e3aec884-a228-4b6d-a532-05fd65087a48</t>
+          <t>87a656f1-8fc2-462a-a53a-073c2b9daed5</t>
         </is>
       </c>
     </row>
@@ -3454,33 +3199,38 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>دولفين</t>
+          <t>دولفين 3</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>1621372</t>
+          <t>255495</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>3976 PSI</t>
+          <t>80 BAR</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I62" s="2" t="n"/>
       <c r="K62" t="inlineStr">
         <is>
-          <t>64997882-0ee1-40a9-915f-755020f5000a</t>
+          <t>058568b7-496b-4985-b337-5837971f8550</t>
         </is>
       </c>
     </row>
@@ -3497,33 +3247,38 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>دولفين</t>
+          <t>دولفين 3</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>1621375</t>
+          <t>258089</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>3976 PSI</t>
+          <t>180 BAR</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I63" s="2" t="n"/>
       <c r="K63" t="inlineStr">
         <is>
-          <t>4277ded0-e1d1-42c0-8785-4cbbb9dd90a5</t>
+          <t>57d0fd34-f65c-4ac2-ba95-11d3308e35da</t>
         </is>
       </c>
     </row>
@@ -3540,33 +3295,38 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>دولفين</t>
+          <t>دولفين 3</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>1709590</t>
+          <t>258251</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>3976 PSI</t>
+          <t>275 BAR</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I64" s="2" t="n"/>
       <c r="K64" t="inlineStr">
         <is>
-          <t>1043c4fb-0f26-4435-8a42-4e8e8c145d82</t>
+          <t>edf09f69-dd8c-4974-af41-b9d9d369a186</t>
         </is>
       </c>
     </row>
@@ -3583,33 +3343,38 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>دولفين</t>
+          <t>دولفين 3</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>264845</t>
+          <t>260341</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>306 BAR</t>
+          <t>18 BAR</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I65" s="2" t="n"/>
       <c r="K65" t="inlineStr">
         <is>
-          <t>d8eccaf9-9f5f-4808-bc4d-0ccf1010900a</t>
+          <t>7cc7410a-2c74-4734-923a-d4e3e9045483</t>
         </is>
       </c>
     </row>
@@ -3626,33 +3391,38 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>دولفين</t>
+          <t>دولفين 3</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>265237</t>
+          <t>262552</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>306 BAR</t>
+          <t>19 BAR</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I66" s="2" t="n"/>
       <c r="K66" t="inlineStr">
         <is>
-          <t>7a5b1fad-63c3-439d-ae58-79f810a75384</t>
+          <t>9a185c16-ec5a-4d34-943d-c848daf636c8</t>
         </is>
       </c>
     </row>
@@ -3669,33 +3439,38 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>دولفين</t>
+          <t>دولفين 3</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>419991</t>
+          <t>262559</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>3976 PSI</t>
+          <t>35 BAR</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I67" s="2" t="n"/>
       <c r="K67" t="inlineStr">
         <is>
-          <t>22e96751-6246-4675-a574-03ea86b3ae6a</t>
+          <t>bf9ccac0-d582-4f7a-b31b-23b52ef3babb</t>
         </is>
       </c>
     </row>
@@ -4192,38 +3967,33 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>دولفين 3</t>
+          <t>دولفين</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>255495</t>
+          <t>1621372</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>80 BAR</t>
+          <t>3976 PSI</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I78" s="2" t="n"/>
       <c r="K78" t="inlineStr">
         <is>
-          <t>058568b7-496b-4985-b337-5837971f8550</t>
+          <t>64997882-0ee1-40a9-915f-755020f5000a</t>
         </is>
       </c>
     </row>
@@ -4240,38 +4010,33 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>دولفين 3</t>
+          <t>دولفين</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>258089</t>
+          <t>1621375</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>180 BAR</t>
+          <t>3976 PSI</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I79" s="2" t="n"/>
       <c r="K79" t="inlineStr">
         <is>
-          <t>57d0fd34-f65c-4ac2-ba95-11d3308e35da</t>
+          <t>4277ded0-e1d1-42c0-8785-4cbbb9dd90a5</t>
         </is>
       </c>
     </row>
@@ -4288,38 +4053,33 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>دولفين 3</t>
+          <t>دولفين</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>258251</t>
+          <t>1709590</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>275 BAR</t>
+          <t>3976 PSI</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I80" s="2" t="n"/>
       <c r="K80" t="inlineStr">
         <is>
-          <t>edf09f69-dd8c-4974-af41-b9d9d369a186</t>
+          <t>1043c4fb-0f26-4435-8a42-4e8e8c145d82</t>
         </is>
       </c>
     </row>
@@ -4336,38 +4096,33 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>دولفين 3</t>
+          <t>دولفين</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>260341</t>
+          <t>264845</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>18 BAR</t>
+          <t>306 BAR</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I81" s="2" t="n"/>
       <c r="K81" t="inlineStr">
         <is>
-          <t>7cc7410a-2c74-4734-923a-d4e3e9045483</t>
+          <t>d8eccaf9-9f5f-4808-bc4d-0ccf1010900a</t>
         </is>
       </c>
     </row>
@@ -4384,38 +4139,33 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>دولفين 3</t>
+          <t>دولفين</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>262552</t>
+          <t>265237</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>19 BAR</t>
+          <t>306 BAR</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I82" s="2" t="n"/>
       <c r="K82" t="inlineStr">
         <is>
-          <t>9a185c16-ec5a-4d34-943d-c848daf636c8</t>
+          <t>7a5b1fad-63c3-439d-ae58-79f810a75384</t>
         </is>
       </c>
     </row>
@@ -4432,38 +4182,33 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>دولفين 3</t>
+          <t>دولفين</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>262559</t>
+          <t>419991</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>35 BAR</t>
+          <t>3976 PSI</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
           <t>الدولفين 1 | الدولفين 2 | الدولفين 3 | الدولفين 4</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>الدولفين 3</t>
         </is>
       </c>
       <c r="I83" s="2" t="n"/>
       <c r="K83" t="inlineStr">
         <is>
-          <t>bf9ccac0-d582-4f7a-b31b-23b52ef3babb</t>
+          <t>22e96751-6246-4675-a574-03ea86b3ae6a</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4461,7 @@
       <c r="I89" s="2" t="n"/>
       <c r="K89" t="inlineStr">
         <is>
-          <t>6f2d73a2-8fa2-4fd4-acb8-0a9a972967f8</t>
+          <t>195f42dc-fa45-4fb4-84da-91b00f2519a0</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4499,7 @@
       <c r="I90" s="2" t="n"/>
       <c r="K90" t="inlineStr">
         <is>
-          <t>195f42dc-fa45-4fb4-84da-91b00f2519a0</t>
+          <t>6f2d73a2-8fa2-4fd4-acb8-0a9a972967f8</t>
         </is>
       </c>
     </row>
@@ -6213,22 +5958,17 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>دائري الهرم 1 فويل أب</t>
+          <t>دائري الهرم فويل أب</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>JTC-2102-119</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>164.8 BAR</t>
+          <t>300 BAR</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -6237,9 +5977,14 @@
         </is>
       </c>
       <c r="I125" s="2" t="n"/>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>مشترك بين الـ 2 Unit — يفضل على المحطة</t>
+        </is>
+      </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>c40bb478-a2a3-47e2-9cbd-49c623dace49</t>
+          <t>533b433c-2d54-4644-9b6c-55cfdc0b8667</t>
         </is>
       </c>
     </row>
@@ -6256,22 +6001,17 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>دائري الهرم 1 فويل أب</t>
+          <t>دائري الهرم فويل أب</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>JTC-2102-185</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>294.2 BAR</t>
+          <t>300 BAR</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -6280,9 +6020,14 @@
         </is>
       </c>
       <c r="I126" s="2" t="n"/>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>مشترك بين الـ 2 Unit — يفضل على المحطة</t>
+        </is>
+      </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>da220da5-66a1-4746-8eb4-9ad12f00a3a1</t>
+          <t>0834470d-8c40-45db-9a61-a49d19383600</t>
         </is>
       </c>
     </row>
@@ -6299,22 +6044,17 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>دائري الهرم 1 فويل أب</t>
+          <t>دائري الهرم فويل أب</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>JTC-2102-246</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>32.4 BAR</t>
+          <t>300 BAR</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -6323,9 +6063,14 @@
         </is>
       </c>
       <c r="I127" s="2" t="n"/>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>مشترك بين الـ 2 Unit — يفضل على المحطة</t>
+        </is>
+      </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>9dd04bce-70df-472a-8d26-e02cd61c562a</t>
+          <t>5a6420bc-e67b-4df9-88a2-3cef0e5d9118</t>
         </is>
       </c>
     </row>
@@ -6337,38 +6082,33 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>دائري الهرم 1 فويل أب</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>JTC-2102-298</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>65.7 BAR</t>
+          <t>300 BAR</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى 1 | فويل اب الدائرى 2</t>
+          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
         </is>
       </c>
       <c r="I128" s="2" t="n"/>
       <c r="K128" t="inlineStr">
         <is>
-          <t>44b404f4-8d53-4945-b6b3-e31346847f06</t>
+          <t>632b667e-da81-4875-b6a6-a1d762bb9664</t>
         </is>
       </c>
     </row>
@@ -6380,38 +6120,33 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>دائري الهرم 1 فويل أب</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>jtc-2102-356</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>17.7 BAR</t>
+          <t>300 BAR</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى 1 | فويل اب الدائرى 2</t>
+          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
         </is>
       </c>
       <c r="I129" s="2" t="n"/>
       <c r="K129" t="inlineStr">
         <is>
-          <t>29db9650-3689-4cdc-bd33-e697caca68ca</t>
+          <t>483ff013-1821-445c-93c1-92bd299b6777</t>
         </is>
       </c>
     </row>
@@ -6423,38 +6158,33 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>دائري الهرم 2 فويل أب</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>JTC-2102-1269</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>17.7 BAR</t>
+          <t>300 BAR</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى 1 | فويل اب الدائرى 2</t>
+          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
         </is>
       </c>
       <c r="I130" s="2" t="n"/>
       <c r="K130" t="inlineStr">
         <is>
-          <t>e15aca98-6d2f-41b5-8274-89503ff4d410</t>
+          <t>eb7743a8-dd47-4e32-9e6b-a4e79939c3a5</t>
         </is>
       </c>
     </row>
@@ -6466,38 +6196,33 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>دائري الهرم 2 فويل أب</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>JTC-2102-1304</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>164.8 BAR</t>
+          <t>300 BAR</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى 1 | فويل اب الدائرى 2</t>
+          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
         </is>
       </c>
       <c r="I131" s="2" t="n"/>
       <c r="K131" t="inlineStr">
         <is>
-          <t>5eac6515-0d03-4c6c-8b5d-e1454d0c4d08</t>
+          <t>56d79278-21dc-4451-97c8-a7bde19f4898</t>
         </is>
       </c>
     </row>
@@ -6509,38 +6234,33 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>دائري الهرم 2 فويل أب</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>JTC-2102-168</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>294.2 BAR</t>
+          <t>300 BAR</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى 1 | فويل اب الدائرى 2</t>
+          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
         </is>
       </c>
       <c r="I132" s="2" t="n"/>
       <c r="K132" t="inlineStr">
         <is>
-          <t>f43aee6e-345f-4997-83aa-56787cf2936d</t>
+          <t>0ec520f8-3001-44ed-82bb-7f9429e4972b</t>
         </is>
       </c>
     </row>
@@ -6552,38 +6272,33 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>دائري الهرم 2 فويل أب</t>
+          <t>مصدق</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>JTC-2102-234</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>32.4 BAR</t>
+          <t>300 BAR</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى 1 | فويل اب الدائرى 2</t>
+          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
         </is>
       </c>
       <c r="I133" s="2" t="n"/>
       <c r="K133" t="inlineStr">
         <is>
-          <t>096b9316-10fb-429a-aff9-a4e51c240b8b</t>
+          <t>6dd944c0-ec4c-486c-bcf9-6a7e83a62169</t>
         </is>
       </c>
     </row>
@@ -6595,38 +6310,38 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى</t>
+          <t>وادى حوف</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>دائري الهرم 2 فويل أب</t>
+          <t>وادي حوف</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>JTC-2102-284</t>
+          <t>1610394</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>65.7 BAR</t>
+          <t>4000 PSI</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى 1 | فويل اب الدائرى 2</t>
+          <t>وادى حوف 1 | وادى حوف 2</t>
         </is>
       </c>
       <c r="I134" s="2" t="n"/>
       <c r="K134" t="inlineStr">
         <is>
-          <t>f943f3cf-948a-4e82-ac1e-1559b6ab1b2f</t>
+          <t>a5b74e6d-c12b-4df7-aab4-c63464ea9930</t>
         </is>
       </c>
     </row>
@@ -6638,12 +6353,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى</t>
+          <t>وادى حوف</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>دائري الهرم فويل أب</t>
+          <t>وادي حوف</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -6651,20 +6366,25 @@
           <t>Storage</t>
         </is>
       </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>1610398</t>
+        </is>
+      </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>300 BAR</t>
+          <t>4000 PSI</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى 1 | فويل اب الدائرى 2</t>
+          <t>وادى حوف 1 | وادى حوف 2</t>
         </is>
       </c>
       <c r="I135" s="2" t="n"/>
       <c r="K135" t="inlineStr">
         <is>
-          <t>533b433c-2d54-4644-9b6c-55cfdc0b8667</t>
+          <t>1a63c634-b6ea-412d-8506-6ed5e77bf8e8</t>
         </is>
       </c>
     </row>
@@ -6676,12 +6396,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى</t>
+          <t>وادى حوف</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>دائري الهرم فويل أب</t>
+          <t>وادي حوف</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -6689,20 +6409,25 @@
           <t>Storage</t>
         </is>
       </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>1610401</t>
+        </is>
+      </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>300 BAR</t>
+          <t>3976 PSI</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى 1 | فويل اب الدائرى 2</t>
+          <t>وادى حوف 1 | وادى حوف 2</t>
         </is>
       </c>
       <c r="I136" s="2" t="n"/>
       <c r="K136" t="inlineStr">
         <is>
-          <t>5a6420bc-e67b-4df9-88a2-3cef0e5d9118</t>
+          <t>2c9d851d-d418-481b-9171-dd0f0347f3b5</t>
         </is>
       </c>
     </row>
@@ -6714,12 +6439,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى</t>
+          <t>وادى حوف</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>دائري الهرم فويل أب</t>
+          <t>وادي حوف</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -6727,20 +6452,25 @@
           <t>Storage</t>
         </is>
       </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>1614525</t>
+        </is>
+      </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>300 BAR</t>
+          <t>4000 PSI</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>فويل اب الدائرى 1 | فويل اب الدائرى 2</t>
+          <t>وادى حوف 1 | وادى حوف 2</t>
         </is>
       </c>
       <c r="I137" s="2" t="n"/>
       <c r="K137" t="inlineStr">
         <is>
-          <t>0834470d-8c40-45db-9a61-a49d19383600</t>
+          <t>fb3dc058-3cfa-498a-839f-a7b9f9c2d6ea</t>
         </is>
       </c>
     </row>
@@ -6752,12 +6482,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>مصدق</t>
+          <t>وادى حوف</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>مصدق</t>
+          <t>وادي حوف</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -6765,20 +6495,25 @@
           <t>Storage</t>
         </is>
       </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>1621373</t>
+        </is>
+      </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>300 BAR</t>
+          <t>3976 PSI</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
+          <t>وادى حوف 1 | وادى حوف 2</t>
         </is>
       </c>
       <c r="I138" s="2" t="n"/>
       <c r="K138" t="inlineStr">
         <is>
-          <t>eb7743a8-dd47-4e32-9e6b-a4e79939c3a5</t>
+          <t>fb38a9af-62b8-49ff-b73e-3f31d56ed972</t>
         </is>
       </c>
     </row>
@@ -6790,12 +6525,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>مصدق</t>
+          <t>وادى حوف</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>مصدق</t>
+          <t>وادي حوف</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -6803,436 +6538,31 @@
           <t>Storage</t>
         </is>
       </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>1646843</t>
+        </is>
+      </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>300 BAR</t>
+          <t>4000 PSI</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
+          <t>وادى حوف 1 | وادى حوف 2</t>
         </is>
       </c>
       <c r="I139" s="2" t="n"/>
       <c r="K139" t="inlineStr">
         <is>
-          <t>483ff013-1821-445c-93c1-92bd299b6777</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>مصدق</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>مصدق</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>300 BAR</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
-        </is>
-      </c>
-      <c r="I140" s="2" t="n"/>
-      <c r="K140" t="inlineStr">
-        <is>
-          <t>632b667e-da81-4875-b6a6-a1d762bb9664</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>مصدق</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>مصدق</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>300 BAR</t>
-        </is>
-      </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
-        </is>
-      </c>
-      <c r="I141" s="2" t="n"/>
-      <c r="K141" t="inlineStr">
-        <is>
-          <t>0ec520f8-3001-44ed-82bb-7f9429e4972b</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>مصدق</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>مصدق</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="F142" t="inlineStr">
-        <is>
-          <t>300 BAR</t>
-        </is>
-      </c>
-      <c r="G142" t="inlineStr">
-        <is>
-          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
-        </is>
-      </c>
-      <c r="I142" s="2" t="n"/>
-      <c r="K142" t="inlineStr">
-        <is>
-          <t>56d79278-21dc-4451-97c8-a7bde19f4898</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>مصدق</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>مصدق</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t>300 BAR</t>
-        </is>
-      </c>
-      <c r="G143" t="inlineStr">
-        <is>
-          <t>مصدق 1 | مصدق 2 | مصدق 3</t>
-        </is>
-      </c>
-      <c r="I143" s="2" t="n"/>
-      <c r="K143" t="inlineStr">
-        <is>
-          <t>6dd944c0-ec4c-486c-bcf9-6a7e83a62169</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>وادى حوف</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>وادي حوف</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>1610394</t>
-        </is>
-      </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>4000 PSI</t>
-        </is>
-      </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>وادى حوف 1 | وادى حوف 2</t>
-        </is>
-      </c>
-      <c r="I144" s="2" t="n"/>
-      <c r="K144" t="inlineStr">
-        <is>
-          <t>a5b74e6d-c12b-4df7-aab4-c63464ea9930</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>وادى حوف</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>وادي حوف</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>1610398</t>
-        </is>
-      </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>4000 PSI</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>وادى حوف 1 | وادى حوف 2</t>
-        </is>
-      </c>
-      <c r="I145" s="2" t="n"/>
-      <c r="K145" t="inlineStr">
-        <is>
-          <t>1a63c634-b6ea-412d-8506-6ed5e77bf8e8</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>وادى حوف</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>وادي حوف</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>1610401</t>
-        </is>
-      </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>3976 PSI</t>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>وادى حوف 1 | وادى حوف 2</t>
-        </is>
-      </c>
-      <c r="I146" s="2" t="n"/>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>2c9d851d-d418-481b-9171-dd0f0347f3b5</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>وادى حوف</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>وادي حوف</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>1614525</t>
-        </is>
-      </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t>4000 PSI</t>
-        </is>
-      </c>
-      <c r="G147" t="inlineStr">
-        <is>
-          <t>وادى حوف 1 | وادى حوف 2</t>
-        </is>
-      </c>
-      <c r="I147" s="2" t="n"/>
-      <c r="K147" t="inlineStr">
-        <is>
-          <t>fb3dc058-3cfa-498a-839f-a7b9f9c2d6ea</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>وادى حوف</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>وادي حوف</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>1621373</t>
-        </is>
-      </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>3976 PSI</t>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>وادى حوف 1 | وادى حوف 2</t>
-        </is>
-      </c>
-      <c r="I148" s="2" t="n"/>
-      <c r="K148" t="inlineStr">
-        <is>
-          <t>fb38a9af-62b8-49ff-b73e-3f31d56ed972</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>وادى حوف</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>وادي حوف</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>1646843</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>4000 PSI</t>
-        </is>
-      </c>
-      <c r="G149" t="inlineStr">
-        <is>
-          <t>وادى حوف 1 | وادى حوف 2</t>
-        </is>
-      </c>
-      <c r="I149" s="2" t="n"/>
-      <c r="K149" t="inlineStr">
-        <is>
           <t>e7ff1b57-1979-4168-96f1-8cd82ef9c2b1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K149"/>
-  <dataValidations count="148">
+  <autoFilter ref="A1:K139"/>
+  <dataValidations count="138">
     <dataValidation sqref="I2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"الشهداء 1,الشهداء 2"</formula1>
     </dataValidation>
@@ -7612,69 +6942,39 @@
       <formula1>"فويل اب الدائرى 1,فويل اب الدائرى 2"</formula1>
     </dataValidation>
     <dataValidation sqref="I128" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"فويل اب الدائرى 1,فويل اب الدائرى 2"</formula1>
+      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
     </dataValidation>
     <dataValidation sqref="I129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"فويل اب الدائرى 1,فويل اب الدائرى 2"</formula1>
+      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
     </dataValidation>
     <dataValidation sqref="I130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"فويل اب الدائرى 1,فويل اب الدائرى 2"</formula1>
+      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
     </dataValidation>
     <dataValidation sqref="I131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"فويل اب الدائرى 1,فويل اب الدائرى 2"</formula1>
+      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
     </dataValidation>
     <dataValidation sqref="I132" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"فويل اب الدائرى 1,فويل اب الدائرى 2"</formula1>
+      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
     </dataValidation>
     <dataValidation sqref="I133" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"فويل اب الدائرى 1,فويل اب الدائرى 2"</formula1>
+      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
     </dataValidation>
     <dataValidation sqref="I134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"فويل اب الدائرى 1,فويل اب الدائرى 2"</formula1>
+      <formula1>"وادى حوف 1,وادى حوف 2"</formula1>
     </dataValidation>
     <dataValidation sqref="I135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"فويل اب الدائرى 1,فويل اب الدائرى 2"</formula1>
+      <formula1>"وادى حوف 1,وادى حوف 2"</formula1>
     </dataValidation>
     <dataValidation sqref="I136" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"فويل اب الدائرى 1,فويل اب الدائرى 2"</formula1>
+      <formula1>"وادى حوف 1,وادى حوف 2"</formula1>
     </dataValidation>
     <dataValidation sqref="I137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"فويل اب الدائرى 1,فويل اب الدائرى 2"</formula1>
+      <formula1>"وادى حوف 1,وادى حوف 2"</formula1>
     </dataValidation>
     <dataValidation sqref="I138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
+      <formula1>"وادى حوف 1,وادى حوف 2"</formula1>
     </dataValidation>
     <dataValidation sqref="I139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"مصدق 1,مصدق 2,مصدق 3"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I144" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"وادى حوف 1,وادى حوف 2"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I145" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"وادى حوف 1,وادى حوف 2"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"وادى حوف 1,وادى حوف 2"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"وادى حوف 1,وادى حوف 2"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"وادى حوف 1,وادى حوف 2"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I149" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"وادى حوف 1,وادى حوف 2"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>